<commit_message>
patrones de comportamiento Strategy, Observer, Command
</commit_message>
<xml_diff>
--- a/LosBichos/ventas.xlsx
+++ b/LosBichos/ventas.xlsx
@@ -41,7 +41,7 @@
     <t>Hamlet - Teatro</t>
   </si>
   <si>
-    <t>2026-05-19T18:59:39.948690600</t>
+    <t>2026-05-20T08:14:30.905117200</t>
   </si>
   <si>
     <t>120000.0</t>
@@ -59,7 +59,7 @@
     <t>Ferxxo en concierto</t>
   </si>
   <si>
-    <t>2026-05-19T18:59:39.941176600</t>
+    <t>2026-05-20T08:14:30.899113300</t>
   </si>
   <si>
     <t>250000.0</t>
@@ -71,16 +71,16 @@
     <t>C004</t>
   </si>
   <si>
-    <t>2026-05-19T18:59:39.957659900</t>
+    <t>2026-05-20T08:14:30.910116900</t>
+  </si>
+  <si>
+    <t>CREADA</t>
   </si>
   <si>
     <t>C003</t>
   </si>
   <si>
     <t>90000.0</t>
-  </si>
-  <si>
-    <t>CREADA</t>
   </si>
 </sst>
 </file>
@@ -205,12 +205,12 @@
         <v>16</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>13</v>
@@ -222,10 +222,10 @@
         <v>9</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>